<commit_message>
Initial commit: Generador de QRs con Streamlit
</commit_message>
<xml_diff>
--- a/codigos.xlsx
+++ b/codigos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\Generación de qrs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E306C300-AD75-4596-B4F5-D4680DAC9703}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FCD7BC8-B98F-4D26-B0CD-63B7249ECD84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6180" yWindow="4185" windowWidth="21600" windowHeight="11295" xr2:uid="{A3E3C54B-40FC-41CD-87B3-E2E3F91B7DE0}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A3E3C54B-40FC-41CD-87B3-E2E3F91B7DE0}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -29,6 +29,9 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
@@ -42,14 +45,14 @@
     <t>codigo</t>
   </si>
   <si>
-    <t>Luis Huapaya</t>
+    <t>ALEX CHAMBI</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -74,22 +77,43 @@
     </font>
     <font>
       <b/>
-      <sz val="9"/>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Lexend"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Lexend"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9D2E9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="11">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -100,21 +124,6 @@
     <border>
       <left style="medium">
         <color rgb="FF000000"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FFCCCCCC"/>
       </left>
       <right style="medium">
         <color rgb="FF000000"/>
@@ -247,31 +256,28 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -281,8 +287,17 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -599,12 +614,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B96241B3-7086-4F0E-B5FE-F53792C9F141}">
   <dimension ref="B1:J103"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col min="3" max="3" width="48.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:10" ht="15.75" thickBot="1">
       <c r="B1" t="s">
         <v>1</v>
       </c>
@@ -612,420 +627,411 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="4">
-        <v>900130</v>
+    <row r="2" spans="2:10" ht="15.75" thickBot="1">
+      <c r="B2" s="14">
+        <v>900139</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="13" t="s">
         <v>2</v>
       </c>
       <c r="J2" s="1"/>
     </row>
-    <row r="3" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="2"/>
-      <c r="C3" s="3"/>
-    </row>
-    <row r="4" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="2"/>
-      <c r="C4" s="3"/>
-    </row>
-    <row r="5" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="2"/>
-      <c r="C5" s="3"/>
-    </row>
-    <row r="6" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="2"/>
-      <c r="C6" s="3"/>
-    </row>
-    <row r="7" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="2"/>
-      <c r="C7" s="3"/>
-    </row>
-    <row r="8" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="2"/>
-      <c r="C8" s="3"/>
-    </row>
-    <row r="9" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="2"/>
-      <c r="C9" s="3"/>
-    </row>
-    <row r="10" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="2"/>
-      <c r="C10" s="3"/>
-    </row>
-    <row r="11" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="2"/>
-      <c r="C11" s="3"/>
-    </row>
-    <row r="12" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="2"/>
-      <c r="C12" s="3"/>
-    </row>
-    <row r="13" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="2"/>
-      <c r="C13" s="3"/>
-    </row>
-    <row r="14" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="2"/>
-      <c r="C14" s="3"/>
-    </row>
-    <row r="15" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="2"/>
-      <c r="C15" s="3"/>
-    </row>
-    <row r="16" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="2"/>
-      <c r="C16" s="3"/>
-    </row>
-    <row r="17" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="2"/>
-      <c r="C17" s="3"/>
-    </row>
-    <row r="18" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="2"/>
-      <c r="C18" s="3"/>
-    </row>
-    <row r="19" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="2"/>
-      <c r="C19" s="3"/>
-    </row>
-    <row r="20" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="2"/>
-      <c r="C20" s="3"/>
-    </row>
-    <row r="21" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="2"/>
-      <c r="C21" s="3"/>
-    </row>
-    <row r="22" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="2"/>
-      <c r="C22" s="3"/>
-    </row>
-    <row r="23" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="2"/>
-      <c r="C23" s="3"/>
-    </row>
-    <row r="24" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="2"/>
-      <c r="C24" s="3"/>
-    </row>
-    <row r="25" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="2"/>
-      <c r="C25" s="3"/>
-    </row>
-    <row r="26" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="2"/>
-      <c r="C26" s="3"/>
-    </row>
-    <row r="27" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="2"/>
-      <c r="C27" s="3"/>
-    </row>
-    <row r="28" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="2"/>
-      <c r="C28" s="3"/>
-    </row>
-    <row r="29" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="2"/>
-      <c r="C29" s="3"/>
-    </row>
-    <row r="30" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="2"/>
-      <c r="C30" s="3"/>
-    </row>
-    <row r="31" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B31" s="2"/>
-      <c r="C31" s="3"/>
-    </row>
-    <row r="32" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="2"/>
-      <c r="C32" s="3"/>
-    </row>
-    <row r="33" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="2"/>
-      <c r="C33" s="3"/>
-    </row>
-    <row r="34" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="2"/>
-      <c r="C34" s="3"/>
-    </row>
-    <row r="35" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="2"/>
-      <c r="C35" s="3"/>
-    </row>
-    <row r="36" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B36" s="2"/>
-      <c r="C36" s="3"/>
-    </row>
-    <row r="37" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B37" s="2"/>
-      <c r="C37" s="3"/>
-    </row>
-    <row r="38" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B38" s="2"/>
-      <c r="C38" s="3"/>
-    </row>
-    <row r="39" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B39" s="2"/>
-      <c r="C39" s="3"/>
-    </row>
-    <row r="40" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B40" s="2"/>
-      <c r="C40" s="3"/>
-    </row>
-    <row r="41" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B41" s="2"/>
-      <c r="C41" s="3"/>
-    </row>
-    <row r="42" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B42" s="2"/>
-      <c r="C42" s="3"/>
-    </row>
-    <row r="43" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B43" s="2"/>
-      <c r="C43" s="3"/>
-    </row>
-    <row r="44" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B44" s="2"/>
-      <c r="C44" s="3"/>
-    </row>
-    <row r="45" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B45" s="2"/>
-      <c r="C45" s="3"/>
-    </row>
-    <row r="46" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B46" s="2"/>
-      <c r="C46" s="3"/>
-    </row>
-    <row r="47" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B47" s="2"/>
-      <c r="C47" s="3"/>
-    </row>
-    <row r="48" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B48" s="2"/>
-      <c r="C48" s="3"/>
-    </row>
-    <row r="49" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B49" s="2"/>
-      <c r="C49" s="3"/>
-    </row>
-    <row r="50" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B50" s="2"/>
-      <c r="C50" s="3"/>
-    </row>
-    <row r="51" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B51" s="2"/>
+    <row r="3" spans="2:10" ht="15.75" thickBot="1">
+      <c r="B3" s="15"/>
+      <c r="C3" s="12"/>
+    </row>
+    <row r="4" spans="2:10" ht="15.75" thickBot="1">
+      <c r="B4" s="14"/>
+      <c r="C4" s="13"/>
+    </row>
+    <row r="5" spans="2:10" ht="15.75" thickBot="1">
+      <c r="B5" s="15"/>
+      <c r="C5" s="12"/>
+    </row>
+    <row r="6" spans="2:10" ht="15.75" thickBot="1">
+      <c r="B6" s="14"/>
+      <c r="C6" s="13"/>
+    </row>
+    <row r="7" spans="2:10" ht="15.75" thickBot="1">
+      <c r="B7" s="15"/>
+      <c r="C7" s="12"/>
+    </row>
+    <row r="8" spans="2:10" ht="15.75" thickBot="1">
+      <c r="B8" s="14"/>
+      <c r="C8" s="13"/>
+    </row>
+    <row r="9" spans="2:10" ht="15.75" thickBot="1">
+      <c r="B9" s="15"/>
+      <c r="C9" s="12"/>
+    </row>
+    <row r="10" spans="2:10" ht="15.75" thickBot="1">
+      <c r="B10" s="14"/>
+      <c r="C10" s="13"/>
+    </row>
+    <row r="11" spans="2:10" ht="15.75" thickBot="1">
+      <c r="B11" s="15"/>
+    </row>
+    <row r="13" spans="2:10" ht="15.75" thickBot="1"/>
+    <row r="14" spans="2:10" ht="15.75" thickBot="1">
+      <c r="C14" s="13"/>
+    </row>
+    <row r="15" spans="2:10" ht="15.75" thickBot="1">
+      <c r="B15" s="15"/>
+      <c r="C15" s="12"/>
+    </row>
+    <row r="16" spans="2:10" ht="15.75" thickBot="1">
+      <c r="B16" s="14"/>
+      <c r="C16" s="13"/>
+    </row>
+    <row r="17" spans="2:3" ht="15.75" thickBot="1">
+      <c r="B17" s="15"/>
+      <c r="C17" s="12"/>
+    </row>
+    <row r="18" spans="2:3" ht="15.75" thickBot="1">
+      <c r="B18" s="15"/>
+      <c r="C18" s="13"/>
+    </row>
+    <row r="19" spans="2:3" ht="15.75" thickBot="1">
+      <c r="B19" s="15"/>
+      <c r="C19" s="12"/>
+    </row>
+    <row r="20" spans="2:3" ht="15.75" thickBot="1">
+      <c r="B20" s="15"/>
+      <c r="C20" s="13"/>
+    </row>
+    <row r="21" spans="2:3" ht="15.75" thickBot="1">
+      <c r="B21" s="15"/>
+      <c r="C21" s="12"/>
+    </row>
+    <row r="22" spans="2:3" ht="15.75" thickBot="1">
+      <c r="B22" s="15"/>
+      <c r="C22" s="13"/>
+    </row>
+    <row r="23" spans="2:3" ht="15.75" thickBot="1">
+      <c r="B23" s="15"/>
+      <c r="C23" s="12"/>
+    </row>
+    <row r="24" spans="2:3" ht="15.75" thickBot="1">
+      <c r="B24" s="15"/>
+      <c r="C24" s="13"/>
+    </row>
+    <row r="25" spans="2:3" ht="15.75" thickBot="1">
+      <c r="B25" s="15"/>
+      <c r="C25" s="12"/>
+    </row>
+    <row r="26" spans="2:3" ht="15.75" thickBot="1">
+      <c r="B26" s="15"/>
+      <c r="C26" s="13"/>
+    </row>
+    <row r="27" spans="2:3" ht="15.75" thickBot="1">
+      <c r="B27" s="15"/>
+      <c r="C27" s="12"/>
+    </row>
+    <row r="28" spans="2:3" ht="15.75" thickBot="1">
+      <c r="B28" s="15"/>
+      <c r="C28" s="13"/>
+    </row>
+    <row r="29" spans="2:3" ht="15.75" thickBot="1">
+      <c r="B29" s="15"/>
+      <c r="C29" s="12"/>
+    </row>
+    <row r="30" spans="2:3" ht="15.75" thickBot="1">
+      <c r="B30" s="15"/>
+      <c r="C30" s="13"/>
+    </row>
+    <row r="31" spans="2:3" ht="15.75" thickBot="1">
+      <c r="B31" s="15"/>
+      <c r="C31" s="12"/>
+    </row>
+    <row r="32" spans="2:3" ht="15.75" thickBot="1">
+      <c r="B32" s="15"/>
+      <c r="C32" s="12"/>
+    </row>
+    <row r="33" spans="2:3" ht="15.75" thickBot="1">
+      <c r="B33" s="15"/>
+      <c r="C33" s="13"/>
+    </row>
+    <row r="34" spans="2:3" ht="15.75" thickBot="1">
+      <c r="B34" s="15"/>
+      <c r="C34" s="12"/>
+    </row>
+    <row r="35" spans="2:3" ht="15.75" thickBot="1">
+      <c r="B35" s="15"/>
+      <c r="C35" s="13"/>
+    </row>
+    <row r="36" spans="2:3" ht="15.75" thickBot="1">
+      <c r="B36" s="15"/>
+      <c r="C36" s="12"/>
+    </row>
+    <row r="37" spans="2:3" ht="15.75" thickBot="1">
+      <c r="B37" s="15"/>
+      <c r="C37" s="13"/>
+    </row>
+    <row r="38" spans="2:3" ht="15.75" thickBot="1">
+      <c r="B38" s="15"/>
+      <c r="C38" s="12"/>
+    </row>
+    <row r="39" spans="2:3" ht="15.75" thickBot="1">
+      <c r="B39" s="15"/>
+      <c r="C39" s="13"/>
+    </row>
+    <row r="40" spans="2:3" ht="15.75" thickBot="1">
+      <c r="B40" s="15"/>
+      <c r="C40" s="12"/>
+    </row>
+    <row r="41" spans="2:3" ht="15.75" thickBot="1">
+      <c r="B41" s="15"/>
+      <c r="C41" s="13"/>
+    </row>
+    <row r="42" spans="2:3" ht="15.75" thickBot="1">
+      <c r="B42" s="15"/>
+      <c r="C42" s="12"/>
+    </row>
+    <row r="43" spans="2:3" ht="15.75" thickBot="1">
+      <c r="B43" s="15"/>
+      <c r="C43" s="13"/>
+    </row>
+    <row r="44" spans="2:3" ht="15.75" thickBot="1">
+      <c r="B44" s="15"/>
+      <c r="C44" s="12"/>
+    </row>
+    <row r="45" spans="2:3" ht="15.75" thickBot="1">
+      <c r="B45" s="15"/>
+      <c r="C45" s="13"/>
+    </row>
+    <row r="46" spans="2:3" ht="15.75" thickBot="1">
+      <c r="B46" s="15"/>
+      <c r="C46" s="12"/>
+    </row>
+    <row r="47" spans="2:3" ht="15.75" thickBot="1">
+      <c r="B47" s="15"/>
+      <c r="C47" s="13"/>
+    </row>
+    <row r="48" spans="2:3" ht="15.75" thickBot="1">
+      <c r="B48" s="15"/>
+      <c r="C48" s="12"/>
+    </row>
+    <row r="49" spans="2:3" ht="15.75" thickBot="1">
+      <c r="B49" s="15"/>
+      <c r="C49" s="12"/>
+    </row>
+    <row r="50" spans="2:3" ht="15.75" thickBot="1">
+      <c r="B50" s="15"/>
+      <c r="C50" s="13"/>
+    </row>
+    <row r="51" spans="2:3" ht="15.75" thickBot="1">
+      <c r="B51" s="15"/>
       <c r="C51" s="3"/>
     </row>
-    <row r="52" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:3" ht="15.75" thickBot="1">
       <c r="B52" s="2"/>
       <c r="C52" s="3"/>
     </row>
-    <row r="53" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:3" ht="15.75" thickBot="1">
       <c r="B53" s="2"/>
       <c r="C53" s="3"/>
     </row>
-    <row r="54" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:3" ht="15.75" thickBot="1">
       <c r="B54" s="2"/>
       <c r="C54" s="3"/>
     </row>
-    <row r="55" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:3" ht="15.75" thickBot="1">
       <c r="B55" s="2"/>
       <c r="C55" s="3"/>
     </row>
-    <row r="56" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:3" ht="15.75" thickBot="1">
       <c r="B56" s="2"/>
       <c r="C56" s="3"/>
     </row>
-    <row r="57" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:3" ht="15.75" thickBot="1">
       <c r="B57" s="2"/>
       <c r="C57" s="3"/>
     </row>
-    <row r="58" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:3" ht="15.75" thickBot="1">
       <c r="B58" s="2"/>
       <c r="C58" s="3"/>
     </row>
-    <row r="59" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:3" ht="15.75" thickBot="1">
       <c r="B59" s="2"/>
       <c r="C59" s="3"/>
     </row>
-    <row r="60" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="2:3" ht="15.75" thickBot="1">
       <c r="B60" s="2"/>
       <c r="C60" s="3"/>
     </row>
-    <row r="61" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="2:3" ht="15.75" thickBot="1">
       <c r="B61" s="2"/>
       <c r="C61" s="3"/>
     </row>
-    <row r="62" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="2:3" ht="15.75" thickBot="1">
       <c r="B62" s="2"/>
       <c r="C62" s="3"/>
     </row>
-    <row r="63" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="2:3" ht="15.75" thickBot="1">
       <c r="B63" s="2"/>
       <c r="C63" s="3"/>
     </row>
-    <row r="64" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="2:3" ht="15.75" thickBot="1">
       <c r="B64" s="2"/>
       <c r="C64" s="3"/>
     </row>
-    <row r="65" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="2:3" ht="15.75" thickBot="1">
       <c r="B65" s="2"/>
       <c r="C65" s="3"/>
     </row>
-    <row r="66" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="2:3" ht="15.75" thickBot="1">
       <c r="B66" s="2"/>
       <c r="C66" s="3"/>
     </row>
-    <row r="67" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="2:3" ht="15.75" thickBot="1">
       <c r="B67" s="2"/>
       <c r="C67" s="3"/>
     </row>
-    <row r="68" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="2:3" ht="15.75" thickBot="1">
       <c r="B68" s="2"/>
       <c r="C68" s="3"/>
     </row>
-    <row r="69" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="2:3" ht="15.75" thickBot="1">
       <c r="B69" s="2"/>
       <c r="C69" s="3"/>
     </row>
-    <row r="70" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="2:3" ht="15.75" thickBot="1">
       <c r="B70" s="2"/>
       <c r="C70" s="3"/>
     </row>
-    <row r="71" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="2:3" ht="15.75" thickBot="1">
       <c r="B71" s="2"/>
       <c r="C71" s="3"/>
     </row>
-    <row r="72" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="2:3" ht="15.75" thickBot="1">
       <c r="B72" s="2"/>
       <c r="C72" s="3"/>
     </row>
-    <row r="73" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="2:3" ht="15.75" thickBot="1">
       <c r="B73" s="2"/>
       <c r="C73" s="3"/>
     </row>
-    <row r="74" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="2:3" ht="15.75" thickBot="1">
       <c r="B74" s="2"/>
       <c r="C74" s="3"/>
     </row>
-    <row r="75" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="2:3" ht="15.75" thickBot="1">
       <c r="B75" s="2"/>
       <c r="C75" s="3"/>
     </row>
-    <row r="76" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="2:3" ht="15.75" thickBot="1">
       <c r="B76" s="2"/>
       <c r="C76" s="3"/>
     </row>
-    <row r="77" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="2:3" ht="15.75" thickBot="1">
       <c r="B77" s="2"/>
       <c r="C77" s="3"/>
     </row>
-    <row r="78" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="2:3" ht="15.75" thickBot="1">
       <c r="B78" s="2"/>
       <c r="C78" s="3"/>
     </row>
-    <row r="79" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="2:3" ht="15.75" thickBot="1">
       <c r="B79" s="2"/>
       <c r="C79" s="3"/>
     </row>
-    <row r="80" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="2:3" ht="15.75" thickBot="1">
       <c r="B80" s="2"/>
       <c r="C80" s="3"/>
     </row>
-    <row r="81" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="2:3" ht="15.75" thickBot="1">
       <c r="B81" s="2"/>
       <c r="C81" s="3"/>
     </row>
-    <row r="82" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="2:3" ht="15.75" thickBot="1">
       <c r="B82" s="2"/>
       <c r="C82" s="3"/>
     </row>
-    <row r="83" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="2:3" ht="15.75" thickBot="1">
       <c r="B83" s="2"/>
       <c r="C83" s="3"/>
     </row>
-    <row r="84" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="2:3" ht="15.75" thickBot="1">
       <c r="B84" s="2"/>
       <c r="C84" s="3"/>
     </row>
-    <row r="85" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="2:3" ht="15.75" thickBot="1">
       <c r="B85" s="2"/>
       <c r="C85" s="3"/>
     </row>
-    <row r="86" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="2:3" ht="15.75" thickBot="1">
       <c r="B86" s="2"/>
       <c r="C86" s="3"/>
     </row>
-    <row r="87" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="2:3" ht="15.75" thickBot="1">
       <c r="B87" s="2"/>
       <c r="C87" s="3"/>
     </row>
-    <row r="88" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="2:3" ht="15.75" thickBot="1">
       <c r="B88" s="2"/>
       <c r="C88" s="3"/>
     </row>
-    <row r="89" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="2:3" ht="15.75" thickBot="1">
       <c r="B89" s="2"/>
       <c r="C89" s="3"/>
     </row>
-    <row r="90" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="2:3" ht="15.75" thickBot="1">
       <c r="B90" s="2"/>
       <c r="C90" s="3"/>
     </row>
-    <row r="91" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="2:3" ht="15.75" thickBot="1">
       <c r="B91" s="2"/>
       <c r="C91" s="3"/>
     </row>
-    <row r="92" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="2:3" ht="15.75" thickBot="1">
       <c r="B92" s="2"/>
       <c r="C92" s="3"/>
     </row>
-    <row r="93" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="2:3" ht="15.75" thickBot="1">
       <c r="B93" s="2"/>
       <c r="C93" s="3"/>
     </row>
-    <row r="94" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="2:3" ht="15.75" thickBot="1">
       <c r="B94" s="2"/>
       <c r="C94" s="3"/>
     </row>
-    <row r="95" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="2:3" ht="15.75" thickBot="1">
       <c r="B95" s="2"/>
       <c r="C95" s="3"/>
     </row>
-    <row r="96" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="2:3" ht="15.75" thickBot="1">
       <c r="B96" s="2"/>
       <c r="C96" s="3"/>
     </row>
-    <row r="97" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="2:3" ht="15.75" thickBot="1">
       <c r="B97" s="2"/>
       <c r="C97" s="3"/>
     </row>
-    <row r="98" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="2:3" ht="15.75" thickBot="1">
       <c r="B98" s="2"/>
-      <c r="C98" s="3"/>
-    </row>
-    <row r="99" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B99" s="6"/>
-      <c r="C99" s="7"/>
-    </row>
-    <row r="100" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B100" s="10"/>
+      <c r="C98" s="5"/>
+    </row>
+    <row r="99" spans="2:3" ht="15.75" thickBot="1">
+      <c r="B99" s="4"/>
+      <c r="C99" s="9"/>
+    </row>
+    <row r="100" spans="2:3" ht="15.75" thickBot="1">
+      <c r="B100" s="8"/>
       <c r="C100" s="11"/>
     </row>
-    <row r="101" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B101" s="12"/>
-      <c r="C101" s="13"/>
-    </row>
-    <row r="102" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B102" s="8"/>
-      <c r="C102" s="8"/>
-    </row>
-    <row r="103" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B103" s="9"/>
-      <c r="C103" s="9"/>
+    <row r="101" spans="2:3" ht="15.75" thickBot="1">
+      <c r="B101" s="10"/>
+      <c r="C101" s="6"/>
+    </row>
+    <row r="102" spans="2:3">
+      <c r="B102" s="6"/>
+      <c r="C102" s="7"/>
+    </row>
+    <row r="103" spans="2:3">
+      <c r="B103" s="7"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="257" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>

</xml_diff>